<commit_message>
[PROGRAMMER] implement Plan48 encounter and enemy runtime
Add canonical encounter/enemy authoring data, deterministic wave/spawn runtime, three typed enemy behaviors, encounter coordination, and v9 save continuity.
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -1,19 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
-    <sheet name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -23,19 +18,17 @@
   <fonts count="3">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="4">
@@ -47,41 +40,35 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F75B5"/>
+        <fgColor rgb="FF2F75B5"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -154,8 +141,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:X7" headerRowCount="1">
-  <autoFilter ref="A3:X7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:X10" headerRowCount="1" totalsRowCount="0">
+  <autoFilter ref="A3:X10"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="Archetype"/>
@@ -187,8 +174,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:X8" headerRowCount="1">
-  <autoFilter ref="A3:X8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:X10" headerRowCount="1" totalsRowCount="0">
+  <autoFilter ref="A3:X10"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="OwnerEnemyId"/>
@@ -299,72 +286,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -420,7 +349,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -429,13 +358,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -469,17 +398,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -534,8 +452,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -545,33 +461,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="27" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" style="3" min="1" max="1"/>
+    <col width="12" customWidth="1" style="3" min="2" max="2"/>
+    <col width="19" customWidth="1" style="3" min="3" max="3"/>
+    <col width="16" customWidth="1" style="3" min="4" max="4"/>
+    <col width="12" customWidth="1" style="3" min="5" max="5"/>
+    <col width="12" customWidth="1" style="3" min="6" max="6"/>
+    <col width="22" customWidth="1" style="3" min="7" max="7"/>
+    <col width="19" customWidth="1" style="3" min="8" max="8"/>
+    <col width="23" customWidth="1" style="3" min="9" max="9"/>
+    <col width="15" customWidth="1" style="3" min="10" max="10"/>
+    <col width="23" customWidth="1" style="3" min="11" max="11"/>
+    <col width="16" customWidth="1" style="3" min="12" max="12"/>
+    <col width="24" customWidth="1" style="3" min="13" max="13"/>
+    <col width="28" customWidth="1" style="3" min="14" max="14"/>
+    <col width="27" customWidth="1" style="3" min="15" max="15"/>
+    <col width="15" customWidth="1" style="3" min="16" max="16"/>
+    <col width="17" customWidth="1" style="3" min="17" max="17"/>
+    <col width="16" customWidth="1" style="3" min="18" max="18"/>
+    <col width="13" customWidth="1" style="3" min="19" max="19"/>
+    <col width="12" customWidth="1" style="3" min="20" max="20"/>
+    <col width="12" customWidth="1" style="3" min="21" max="21"/>
+    <col width="13" customWidth="1" style="3" min="22" max="22"/>
+    <col width="12" customWidth="1" style="3" min="23" max="23"/>
+    <col width="12" customWidth="1" style="3" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -704,490 +620,760 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>M_Grunt</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Grunt</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Enemy.Grunt</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Enemy.Grunt</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>95</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>51.84</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>183.6</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>0.22</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>360</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>怪物体系M</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="X4" s="3" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>基础近战怪</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>M_Shield</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Shield</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Enemy.Shield</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Enemy.Shield</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>51.84</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>183.6</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>0.22</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>360</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="U5" s="3" t="inlineStr">
+      <c r="U5" s="4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="V5" s="3" t="inlineStr">
+      <c r="V5" s="4" t="inlineStr">
         <is>
           <t>怪物体系M</t>
         </is>
       </c>
-      <c r="W5" s="3" t="inlineStr">
+      <c r="W5" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="X5" s="3" t="inlineStr">
+      <c r="X5" s="4" t="inlineStr">
         <is>
           <t>正面减伤盾怪</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>M_Bomber</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Bomber</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Enemy.Bomber</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Enemy.Bomber</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>175</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>51.84</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>183.6</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>0.22</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>360</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>260</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>180</t>
         </is>
       </c>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="T6" s="3" t="inlineStr">
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="U6" s="3" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="V6" s="3" t="inlineStr">
+      <c r="V6" s="4" t="inlineStr">
         <is>
           <t>怪物体系M</t>
         </is>
       </c>
-      <c r="W6" s="3" t="inlineStr">
+      <c r="W6" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="X6" s="3" t="inlineStr">
+      <c r="X6" s="4" t="inlineStr">
         <is>
           <t>接近后引爆</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Boss</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Boss.TimeGuard</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Enemy.TimeGuard</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>650</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>183.6</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>0.22</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>140</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="U7" s="3" t="inlineStr">
+      <c r="U7" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="V7" s="3" t="inlineStr">
+      <c r="V7" s="4" t="inlineStr">
         <is>
           <t>怪物体系M</t>
         </is>
       </c>
-      <c r="W7" s="3" t="inlineStr">
+      <c r="W7" s="4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="X7" s="3" t="inlineStr">
+      <c r="X7" s="4" t="inlineStr">
         <is>
           <t>第六场时间守卫Boss</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Slime</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.Slime</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.Slime</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>190</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>360</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="X8" s="4" t="inlineStr">
+        <is>
+          <t>开普勒近战史莱姆；接触攻击</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.Ranged</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.Rabbit</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>165</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>650</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>360</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="U9" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="X9" s="4" t="inlineStr">
+        <is>
+          <t>开普勒远程兔子；锁定位置范围攻击</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.Elite</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.Fox</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>360</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="X10" s="4" t="inlineStr">
+        <is>
+          <t>开普勒精英狐狸；正面防御与直线突进</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1382,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:X1"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="15">
     <dataValidation sqref="B4:B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Grunt,Shield,Bomber,Boss"</formula1>
     </dataValidation>
@@ -1212,8 +1398,38 @@
     <dataValidation sqref="U4:U7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
+    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Grunt,Shield,Bomber,Boss,Slime,Ranged,Elite"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Boss.TimeGuard,Enemy.Slime,Enemy.Ranged,Enemy.Elite"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D4:D10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Enemy.TimeGuard,Enemy.Slime,Enemy.Rabbit,Enemy.Fox"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U4:U10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Grunt,Shield,Bomber,Boss,Slime,Ranged,Elite"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Boss.TimeGuard,Enemy.Slime,Enemy.Ranged,Enemy.Elite"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D4:D10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Enemy.TimeGuard,Enemy.Slime,Enemy.Rabbit,Enemy.Fox"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U4:U10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -1226,33 +1442,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" style="3" min="1" max="1"/>
+    <col width="14" customWidth="1" style="3" min="2" max="2"/>
+    <col width="12" customWidth="1" style="3" min="3" max="3"/>
+    <col width="15" customWidth="1" style="3" min="4" max="4"/>
+    <col width="12" customWidth="1" style="3" min="5" max="5"/>
+    <col width="12" customWidth="1" style="3" min="6" max="6"/>
+    <col width="15" customWidth="1" style="3" min="7" max="7"/>
+    <col width="15" customWidth="1" style="3" min="8" max="8"/>
+    <col width="17" customWidth="1" style="3" min="9" max="9"/>
+    <col width="17" customWidth="1" style="3" min="10" max="10"/>
+    <col width="12" customWidth="1" style="3" min="11" max="11"/>
+    <col width="12" customWidth="1" style="3" min="12" max="12"/>
+    <col width="12" customWidth="1" style="3" min="13" max="13"/>
+    <col width="12" customWidth="1" style="3" min="14" max="14"/>
+    <col width="12" customWidth="1" style="3" min="15" max="15"/>
+    <col width="28" customWidth="1" style="3" min="16" max="16"/>
+    <col width="18" customWidth="1" style="3" min="17" max="17"/>
+    <col width="15" customWidth="1" style="3" min="18" max="18"/>
+    <col width="12" customWidth="1" style="3" min="19" max="19"/>
+    <col width="24" customWidth="1" style="3" min="20" max="20"/>
+    <col width="17" customWidth="1" style="3" min="21" max="21"/>
+    <col width="13" customWidth="1" style="3" min="22" max="22"/>
+    <col width="12" customWidth="1" style="3" min="23" max="23"/>
+    <col width="12" customWidth="1" style="3" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1385,612 +1601,792 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard_MeleeSweep</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Boss.MeleeSweep</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>0.65</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>0.12</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>0.75</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>2.8</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>260</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>220</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>260</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>LockedDirection</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>WindupStart</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>Boss技能</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="X4" s="3" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr">
         <is>
           <t>近身扇形挥击</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard_Projectile</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Boss.Projectile</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>0.55</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>300</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>1100</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>700</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
         <is>
           <t>LockedLocation</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="S5" s="4" t="inlineStr">
         <is>
           <t>WindupEnd</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V5" s="3" t="inlineStr">
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
         <is>
           <t>Boss技能</t>
         </is>
       </c>
-      <c r="W5" s="3" t="inlineStr">
+      <c r="W5" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="X5" s="3" t="inlineStr">
+      <c r="X5" s="4" t="inlineStr">
         <is>
           <t>不追踪远程投射</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard_BlinkSlam</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Boss.BlinkSlam</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>0.35</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>1100</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>180</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>180</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>LockedLocation</t>
         </is>
       </c>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>WindupStart</t>
         </is>
       </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V6" s="3" t="inlineStr">
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U6" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="inlineStr">
         <is>
           <t>Boss技能</t>
         </is>
       </c>
-      <c r="W6" s="3" t="inlineStr">
+      <c r="W6" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="X6" s="3" t="inlineStr">
+      <c r="X6" s="4" t="inlineStr">
         <is>
           <t>消失后在锁定落点外闪现砸地</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard_PrayerBeam</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Boss.PrayerBeam</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>0.15</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>1200</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>160</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>1200</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t>LockedDirection</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="S7" s="4" t="inlineStr">
         <is>
           <t>WindupEnd</t>
         </is>
       </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
         <is>
           <t>Boss技能</t>
         </is>
       </c>
-      <c r="W7" s="3" t="inlineStr">
+      <c r="W7" s="4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="X7" s="3" t="inlineStr">
+      <c r="X7" s="4" t="inlineStr">
         <is>
           <t>锁定方向长直线光束</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard_ElementCleanse</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Boss.ElementCleanse</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q8" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
         <is>
           <t>Self</t>
         </is>
       </c>
-      <c r="S8" s="3" t="inlineStr">
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>Interval</t>
         </is>
       </c>
-      <c r="T8" s="3" t="inlineStr">
+      <c r="T8" s="4" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="U8" s="3" t="inlineStr">
+      <c r="U8" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V8" s="3" t="inlineStr">
+      <c r="V8" s="4" t="inlineStr">
         <is>
           <t>Boss技能</t>
         </is>
       </c>
-      <c r="W8" s="3" t="inlineStr">
+      <c r="W8" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="X8" s="3" t="inlineStr">
+      <c r="X8" s="4" t="inlineStr">
         <is>
           <t>定时清除元素并获得短暂免疫</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_RangedBurst</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.RangedBurst</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>LockedLocation</t>
+        </is>
+      </c>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="4" t="inlineStr">
+        <is>
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="X9" s="4" t="inlineStr">
+        <is>
+          <t>锁定落点；半径1.5m；每技能冷却2s</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_Dash</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.EliteDash</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>LockedDirection</t>
+        </is>
+      </c>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="X10" s="4" t="inlineStr">
+        <is>
+          <t>预警0.8s；长4.5m宽1.4m；冷却4s</t>
         </is>
       </c>
     </row>
@@ -1999,7 +2395,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:X1"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="15">
     <dataValidation sqref="C4:C8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse"</formula1>
     </dataValidation>
@@ -2015,8 +2411,38 @@
     <dataValidation sqref="B4:B8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
+    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>INDIRECT("tblEnemies[Id]")</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse,Enemy.RangedBurst,Enemy.EliteDash"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"LockedLocation,LockedDirection,Self"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S4:S10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"WindupStart,WindupEnd,Interval"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>INDIRECT("tblEnemies[Id]")</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse,Enemy.RangedBurst,Enemy.EliteDash"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"LockedLocation,LockedDirection,Self"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S4:S10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"WindupStart,WindupEnd,Interval"</formula1>
+    </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -2032,20 +2458,20 @@
   <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" style="3" min="1" max="1"/>
+    <col width="13" customWidth="1" style="3" min="2" max="2"/>
+    <col width="12" customWidth="1" style="3" min="3" max="3"/>
+    <col width="16" customWidth="1" style="3" min="4" max="4"/>
+    <col width="12" customWidth="1" style="3" min="5" max="5"/>
+    <col width="26" customWidth="1" style="3" min="6" max="6"/>
+    <col width="27" customWidth="1" style="3" min="7" max="7"/>
+    <col width="23" customWidth="1" style="3" min="8" max="8"/>
+    <col width="25" customWidth="1" style="3" min="9" max="9"/>
+    <col width="20" customWidth="1" style="3" min="10" max="10"/>
+    <col width="12" customWidth="1" style="3" min="11" max="11"/>
+    <col width="13" customWidth="1" style="3" min="12" max="12"/>
+    <col width="12" customWidth="1" style="3" min="13" max="13"/>
+    <col width="12" customWidth="1" style="3" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2128,72 +2554,72 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard_ThirtySeconds</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>M_TimeGuard</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>DestroyEncounterEchoes</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>1.25</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Boss阶段</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>仅局内一次性强化且不回血不改最大生命</t>
         </is>
@@ -2204,7 +2630,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="12">
     <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"DestroyEncounterEchoes"</formula1>
     </dataValidation>
@@ -2217,8 +2643,32 @@
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>INDIRECT("tblEnemies[Id]")</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"None,RetireEncounterEchoes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"None,RefillToMaximum"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>INDIRECT("tblEnemies[Id]")</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"None,RetireEncounterEchoes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"None,RefillToMaximum"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -2234,11 +2684,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" style="3" min="1" max="1"/>
+    <col width="28" customWidth="1" style="3" min="2" max="2"/>
+    <col width="28" customWidth="1" style="3" min="3" max="3"/>
+    <col width="28" customWidth="1" style="3" min="4" max="4"/>
+    <col width="28" customWidth="1" style="3" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2339,7 +2789,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
[PROGRAMMER] Plan 68 WS1: 怪物系统对齐 - 数据模型地基
新增按场次数值成长与双形态触发的数据模型，对齐怪物.xlsx 权威源。

- csv_schema.csv: Enemies 加 4 个双形态列(Phase2Enabled/Phase2TriggerRangeCm/Phase2RequiredAttackCount/Phase2TransformSeconds)，新增 EnemyCombatStats 表。
- reecho_data_manifest.csv: 注册 enemy_combat_stats.csv 白名单。
- ReEchoEnemyData.xlsx: Enemies 表加 4 列(SLIME/RABBIT/FOX 填权威触发值)，新建 EnemyCombatStats 表(24 行成长数据)，_ExportMap 加行。
- sync_xlsx_to_csv.py + validate_project.py: 注册新表与列(CSV_TABLES / TABLE_TO_CSV)。
- C++: FReEchoCsvEnemyRow 加 Phase2 字段；新增 FReEchoCsvEnemyCombatStatRow；Snapshot 加 EnemyCombatStats 映射与 FindEnemyCombatStat 访问器；ReadEnemies 读双形态列；新增 ReadEnemyCombatStats 并在 ReadTables 接线。
- 随附增量构建刷新的 prebuilt 包。

WS1 仅数据模型，未改运行时逻辑；双形态/成长的消费在 WS2/WS3。
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -1,12 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="EnemyCombatStats" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -15,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -29,6 +30,9 @@
     <font>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -55,7 +59,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -65,6 +69,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -141,7 +146,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:X10" headerRowCount="1" totalsRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:AB10" headerRowCount="1" totalsRowCount="0">
   <autoFilter ref="A3:X10"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Id"/>
@@ -230,7 +235,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblExportMap" displayName="tblExportMap" ref="A1:E4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblExportMap" displayName="tblExportMap" ref="A1:E5" headerRowCount="1">
   <autoFilter ref="A1:E4"/>
   <tableColumns count="5">
     <tableColumn id="1" name="SheetName"/>
@@ -240,6 +245,21 @@
     <tableColumn id="5" name="SortKey"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblEnemyCombatStats" displayName="tblEnemyCombatStats" ref="A3:F27" headerRowCount="1">
+  <autoFilter ref="A3:F27"/>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="2" name="EnemyId"/>
+    <tableColumn id="3" name="CombatIndex"/>
+    <tableColumn id="4" name="MaxHealth"/>
+    <tableColumn id="5" name="ContactDamage"/>
+    <tableColumn id="6" name="AttackIntervalSeconds"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -461,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -618,6 +638,26 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>Phase2Enabled</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>Phase2TriggerRangeCm</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>Phase2RequiredAttackCount</t>
+        </is>
+      </c>
+      <c r="AB3" s="5" t="inlineStr">
+        <is>
+          <t>Phase2TransformSeconds</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -740,6 +780,18 @@
           <t>基础近战怪</t>
         </is>
       </c>
+      <c r="Y4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -862,6 +914,18 @@
           <t>正面减伤盾怪</t>
         </is>
       </c>
+      <c r="Y5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -984,6 +1048,18 @@
           <t>接近后引爆</t>
         </is>
       </c>
+      <c r="Y6" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1106,6 +1182,18 @@
           <t>第六场时间守卫Boss</t>
         </is>
       </c>
+      <c r="Y7" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1196,6 +1284,18 @@
           <t>开普勒近战史莱姆；接触攻击</t>
         </is>
       </c>
+      <c r="Y8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="AA8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB8" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1286,6 +1386,18 @@
           <t>开普勒远程兔子；锁定位置范围攻击</t>
         </is>
       </c>
+      <c r="Y9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AA9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB9" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1375,6 +1487,18 @@
         <is>
           <t>开普勒精英狐狸；正面防御与直线突进</t>
         </is>
+      </c>
+      <c r="Y10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="AA10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB10" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1437,7 +1561,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1748,7 +1872,7 @@
           <t>true</t>
         </is>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1868,7 +1992,7 @@
           <t>true</t>
         </is>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1988,7 +2112,7 @@
           <t>true</t>
         </is>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -2228,7 +2352,7 @@
           <t>true</t>
         </is>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="4" t="n">
@@ -2438,7 +2562,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2675,7 +2799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="3" min="1" max="1"/>
@@ -2781,6 +2905,29 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EnemyCombatStats</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tblEnemyCombatStats</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>enemy_combat_stats.csv</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2788,4 +2935,639 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF00B0F0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>EnemyCombatStats production table - edit data rows only</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>EnemyId</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>CombatIndex</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>MaxHealth</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>ContactDamage</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>AttackIntervalSeconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C4</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C5</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C6</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C7</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME_C8</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C1</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C2</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C3</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C4</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C5</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C6</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C7</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_C8</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C1</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C2</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C3</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C4</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C5</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C6</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C7</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>176</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX_C8</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[PROGRAMMER] Plan68 WS4+WS5: SHEEP two-phase boss and idle-wander aggro state machine
WS4 (SHEEP boss): add M_SHEEP enemy + 5 abilities, two-phase boss_phases with PhaseMaxHealth refill-to-maximum (3900) on Echo-retire trigger, encounter wave -> M_SHEEP; relax HasExactColumns schema to accept PhaseMaxHealth column.

WS5 (idle wander): FReEchoEnemySenseSnapshot gains bInCombat/HateRangeCm injected by Host; LogicComponent AdvanceIdleWander emits deterministic (WorldTime+SpawnIndex) wander when not engaged; ReEchoEnemyActor injects per-kind aggro radius; once engaged, disengage idles without re-wander. Adds IdleWander automation test. Refreshes prebuilt editor bundle.
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:AB10" headerRowCount="1" totalsRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:AB11" headerRowCount="1" totalsRowCount="0">
   <autoFilter ref="A3:X10"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Id"/>
@@ -179,8 +179,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:X10" headerRowCount="1" totalsRowCount="0">
-  <autoFilter ref="A3:X10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:X15" headerRowCount="1" totalsRowCount="0">
+  <autoFilter ref="A3:X15"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="OwnerEnemyId"/>
@@ -212,9 +212,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblBossPhases" displayName="tblBossPhases" ref="A3:N4" headerRowCount="1">
-  <autoFilter ref="A3:N4"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblBossPhases" displayName="tblBossPhases" ref="A3:O5" headerRowCount="1">
+  <autoFilter ref="A3:O5"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="BossEnemyId"/>
     <tableColumn id="3" name="PhaseIndex"/>
@@ -229,6 +229,7 @@
     <tableColumn id="12" name="SourceSheet"/>
     <tableColumn id="13" name="SourceRow"/>
     <tableColumn id="14" name="Notes"/>
+    <tableColumn id="15" name="PhaseMaxHealth"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -481,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AB11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -1501,6 +1502,140 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Boss.TimeGuard</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.Sheep</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>2600</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>183.6</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>0.22</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="X11" s="4" t="inlineStr">
+        <is>
+          <t>SHEEP two-phase boss</t>
+        </is>
+      </c>
+      <c r="Y11" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
@@ -1522,34 +1657,34 @@
     <dataValidation sqref="U4:U7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Grunt,Shield,Bomber,Boss,Slime,Ranged,Elite"</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="C4:C11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Boss.TimeGuard,Enemy.Slime,Enemy.Ranged,Enemy.Elite"</formula1>
     </dataValidation>
-    <dataValidation sqref="D4:D10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="D4:D11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Enemy.TimeGuard,Enemy.Slime,Enemy.Rabbit,Enemy.Fox"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="U4:U11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Grunt,Shield,Bomber,Boss,Slime,Ranged,Elite"</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="C4:C11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Boss.TimeGuard,Enemy.Slime,Enemy.Ranged,Enemy.Elite"</formula1>
     </dataValidation>
-    <dataValidation sqref="D4:D10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="D4:D11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Enemy.Grunt,Enemy.Shield,Enemy.Bomber,Enemy.TimeGuard,Enemy.Slime,Enemy.Rabbit,Enemy.Fox"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="U4:U11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1566,7 +1701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -2508,6 +2643,616 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP_MeleeSweep</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Boss.MeleeSweep</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>LockedDirection</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="W11" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="X11" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP_Projectile</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Boss.Projectile</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>LockedLocation</t>
+        </is>
+      </c>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>WindupEnd</t>
+        </is>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="W12" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="X12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP_BlinkSlam</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Boss.BlinkSlam</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>LockedLocation</t>
+        </is>
+      </c>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="W13" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="X13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP_PrayerBeam</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Boss.PrayerBeam</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>LockedDirection</t>
+        </is>
+      </c>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>WindupEnd</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="W14" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="X14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP_ElementCleanse</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Boss.ElementCleanse</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>Interval</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V15" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="W15" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="X15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
@@ -2529,34 +3274,34 @@
     <dataValidation sqref="B4:B8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="C4:C15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse,Enemy.RangedBurst,Enemy.EliteDash"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="R4:R10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="R4:R15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"LockedLocation,LockedDirection,Self"</formula1>
     </dataValidation>
-    <dataValidation sqref="S4:S10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="S4:S15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"WindupStart,WindupEnd,Interval"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="C4:C15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse,Enemy.RangedBurst,Enemy.EliteDash"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="R4:R10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="R4:R15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"LockedLocation,LockedDirection,Self"</formula1>
     </dataValidation>
-    <dataValidation sqref="S4:S10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="S4:S15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"WindupStart,WindupEnd,Interval"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2573,7 +3318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -2590,6 +3335,7 @@
     <col width="13" customWidth="1" style="3" min="12" max="12"/>
     <col width="12" customWidth="1" style="3" min="13" max="13"/>
     <col width="12" customWidth="1" style="3" min="14" max="14"/>
+    <col width="12" customWidth="1" style="3" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2670,6 +3416,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>PhaseMaxHealth</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -2740,49 +3491,131 @@
       <c r="N4" s="4" t="inlineStr">
         <is>
           <t>仅局内一次性强化且不回血不改最大生命</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP_Phase1</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>DestroyEncounterEchoes</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>1.4286</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>RefillToMaximum</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>SHEEP two-phase 30s trigger player x1.5 dmg x0.7 cooldown boss max HP plus 1300 and refill</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>3900</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <dataValidations count="12">
-    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"DestroyEncounterEchoes"</formula1>
     </dataValidation>
-    <dataValidation sqref="J4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="J4:J5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"None,RefillToMaximum"</formula1>
     </dataValidation>
-    <dataValidation sqref="K4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="K4:K5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"None,RetireEncounterEchoes"</formula1>
     </dataValidation>
-    <dataValidation sqref="J4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="J4:J5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"None,RefillToMaximum"</formula1>
     </dataValidation>
-    <dataValidation sqref="K4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="K4:K5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"None,RetireEncounterEchoes"</formula1>
     </dataValidation>
-    <dataValidation sqref="J4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="J4:J5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"None,RefillToMaximum"</formula1>
     </dataValidation>
-    <dataValidation sqref="K4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="K4:K5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
[PROGRAMMER] Plan68: make enemy aggro/sensing range (HateRangeCm) data-driven from planner monster workbook; retire hardcoded resolver
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:AD10" headerRowCount="1" totalsRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:AE10" headerRowCount="1" totalsRowCount="0">
   <autoFilter ref="A3:X10"/>
   <tableColumns count="30">
     <tableColumn id="1" name="Id"/>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD10"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -681,6 +681,11 @@
           <t>Phase2HealthThresholdRatio</t>
         </is>
       </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>HateRangeCm</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -789,6 +794,9 @@
       <c r="AD4" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="AE4" s="4" t="n">
+        <v>520</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -897,6 +905,9 @@
       <c r="AD5" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="AE5" s="4" t="n">
+        <v>520</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1005,6 +1016,9 @@
       <c r="AD6" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="AE6" s="4" t="n">
+        <v>520</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1117,6 +1131,9 @@
       <c r="AD7" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="AE7" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1223,6 +1240,9 @@
       <c r="AD8" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="AE8" s="4" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1329,6 +1349,9 @@
       <c r="AD9" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="AE9" s="4" t="n">
+        <v>1500</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1434,6 +1457,9 @@
       <c r="AC10" s="4" t="n"/>
       <c r="AD10" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="AE10" s="4" t="n">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>
@@ -1537,7 +1563,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
[PROGRAMMER] Plan68: non-boss align to planner monster workbook (HP/contact/Phase2) + RABBIT RB_01B; publish csv + refresh prebuilt
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:X10" headerRowCount="1" totalsRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:X11" headerRowCount="1" totalsRowCount="0">
   <autoFilter ref="A3:X10"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Id"/>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0.8</v>
@@ -1157,7 +1157,7 @@
         <v>90</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>1.3</v>
@@ -1207,10 +1207,8 @@
           <t>开普勒近战史莱姆；接触攻击</t>
         </is>
       </c>
-      <c r="Y8" s="4" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="Y8" s="4" t="b">
+        <v>0</v>
       </c>
       <c r="Z8" s="4" t="n">
         <v>2000</v>
@@ -1253,7 +1251,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>0.7</v>
@@ -1265,7 +1263,7 @@
         <v>85</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>2</v>
@@ -1315,10 +1313,8 @@
           <t>开普勒远程兔子；锁定位置范围攻击</t>
         </is>
       </c>
-      <c r="Y9" s="4" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="Y9" s="4" t="b">
+        <v>0</v>
       </c>
       <c r="Z9" s="4" t="n">
         <v>1500</v>
@@ -1361,7 +1357,7 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>1.2</v>
@@ -1373,7 +1369,7 @@
         <v>130</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>4</v>
@@ -1423,10 +1419,8 @@
           <t>开普勒精英狐狸；正面防御与直线突进</t>
         </is>
       </c>
-      <c r="Y10" s="4" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="Y10" s="4" t="b">
+        <v>0</v>
       </c>
       <c r="Z10" s="4" t="n">
         <v>2000</v>
@@ -1507,7 +1501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -1543,6 +1537,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2292,6 +2287,94 @@
       <c r="X10" s="4" t="inlineStr">
         <is>
           <t>预警0.8s；长4.5m宽1.4m；冷却4s</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT_MovingVolley</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Enemy.RangedBurst</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>1080</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>LockedDirection</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>全怪物技能表</t>
+        </is>
+      </c>
+      <c r="W11" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="X11" s="4" t="inlineStr">
+        <is>
+          <t>移动散射(3发)</t>
         </is>
       </c>
     </row>
@@ -2301,49 +2384,49 @@
     <mergeCell ref="A1:X1"/>
   </mergeCells>
   <dataValidations count="15">
-    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="C4:C11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="R4:R10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="R4:R11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"LockedLocation,LockedDirection,Self"</formula1>
     </dataValidation>
-    <dataValidation sqref="S4:S10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="S4:S11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"WindupStart,WindupEnd,Interval"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="C4:C11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse,Enemy.RangedBurst,Enemy.EliteDash"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="R4:R10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="R4:R11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"LockedLocation,LockedDirection,Self"</formula1>
     </dataValidation>
-    <dataValidation sqref="S4:S10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="S4:S11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"WindupStart,WindupEnd,Interval"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="B4:B11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblEnemies[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="C4:C11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse,Enemy.RangedBurst,Enemy.EliteDash"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="E4:E11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="R4:R10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="R4:R11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"LockedLocation,LockedDirection,Self"</formula1>
     </dataValidation>
-    <dataValidation sqref="S4:S10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="S4:S11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"WindupStart,WindupEnd,Interval"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2843,7 +2926,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>2</v>
@@ -2867,7 +2950,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>2</v>
@@ -2891,10 +2974,10 @@
         <v>3</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>1.3</v>
@@ -2915,7 +2998,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>3</v>
@@ -2939,10 +3022,10 @@
         <v>5</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>1.2</v>
@@ -2963,7 +3046,7 @@
         <v>6</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>4</v>
@@ -2987,10 +3070,10 @@
         <v>7</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>1.1</v>
@@ -3011,10 +3094,10 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>1.1</v>
@@ -3035,7 +3118,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>1</v>
@@ -3059,7 +3142,7 @@
         <v>2</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>1</v>
@@ -3083,7 +3166,7 @@
         <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>1</v>
@@ -3107,10 +3190,10 @@
         <v>4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>1.8</v>
@@ -3131,7 +3214,7 @@
         <v>5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>2</v>
@@ -3155,10 +3238,10 @@
         <v>6</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>1.7</v>
@@ -3179,10 +3262,10 @@
         <v>7</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>1.7</v>
@@ -3203,10 +3286,10 @@
         <v>8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>1.6</v>
@@ -3227,7 +3310,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>3</v>
@@ -3251,7 +3334,7 @@
         <v>2</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>3</v>
@@ -3275,7 +3358,7 @@
         <v>3</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>4</v>
@@ -3299,7 +3382,7 @@
         <v>4</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>4</v>
@@ -3323,7 +3406,7 @@
         <v>5</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>118</v>
+        <v>59</v>
       </c>
       <c r="E24" s="4" t="n">
         <v>5</v>
@@ -3347,7 +3430,7 @@
         <v>6</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>146</v>
+        <v>73</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>5</v>
@@ -3371,7 +3454,7 @@
         <v>7</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>176</v>
+        <v>88</v>
       </c>
       <c r="E26" s="4" t="n">
         <v>6</v>
@@ -3395,7 +3478,7 @@
         <v>8</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>220</v>
+        <v>110</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
[PROGRAMMER] Plan68: make enemy projectile volley data-driven (ProjectileCount/SpreadAngleDegrees/bMovementDuringCast) and implement N-projectile fan scatter behavior; fix rabbit test tuning + stale boss-phase validator
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -191,7 +191,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:X11" headerRowCount="1" totalsRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblEnemyAbilities" displayName="tblEnemyAbilities" ref="A3:AA11" headerRowCount="1" totalsRowCount="0">
   <autoFilter ref="A3:X10"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Id"/>
@@ -1527,7 +1527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -1684,8 +1684,23 @@
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="4">
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>ProjectileCount</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>SpreadAngleDegrees</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>bMovementDuringCast</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" s="3">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>M_SHEEP_MeleeSweep</t>
@@ -1774,8 +1789,17 @@
           <t>平A近战挥击；半径3m圆；触发距离2m；二阶段伤害x1.5</t>
         </is>
       </c>
-    </row>
-    <row r="5">
+      <c r="Y4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" s="3">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>M_SHEEP_StationaryVolley</t>
@@ -1864,8 +1888,17 @@
           <t>站定连射4连法杖弹；半径1.5m/射程12m；单发5伤总计20；二阶段总伤30</t>
         </is>
       </c>
-    </row>
-    <row r="6">
+      <c r="Y5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" s="3">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>M_SHEEP_MovingSpread</t>
@@ -1954,8 +1987,17 @@
           <t>移动散射3向法杖弹；半径1.5m/射程12m；单发5伤总计15；二阶段总伤22.5</t>
         </is>
       </c>
-    </row>
-    <row r="7">
+      <c r="Y6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA6" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" s="3">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>M_SHEEP_BlinkSlam</t>
@@ -2044,8 +2086,17 @@
           <t>闪身打击Blink Strike；位移+范围下砸；30伤；二阶段45伤</t>
         </is>
       </c>
-    </row>
-    <row r="8">
+      <c r="Y7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" s="3">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>M_SHEEP_PrayerBeam</t>
@@ -2134,11 +2185,20 @@
           <t>祷告光束Prayer Beam；锁定方向范围攻击；半径5m/射程20m；20伤/次；冷却未定义取默认13s</t>
         </is>
       </c>
-    </row>
-    <row r="9">
+      <c r="Y8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" s="3">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>M_RABBIT_RangedBurst</t>
+          <t>M_RABBIT_MovingVolley</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -2154,10 +2214,8 @@
       <c r="D9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="E9" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>1</v>
@@ -2172,13 +2230,13 @@
         <v>0</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>1000</v>
+        <v>1080</v>
       </c>
       <c r="M9" s="4" t="n">
         <v>150</v>
@@ -2197,7 +2255,7 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>LockedLocation</t>
+          <t>LockedDirection</t>
         </is>
       </c>
       <c r="S9" s="4" t="inlineStr">
@@ -2213,19 +2271,28 @@
       </c>
       <c r="V9" s="4" t="inlineStr">
         <is>
-          <t>怪物配置表</t>
+          <t>全怪物技能表</t>
         </is>
       </c>
       <c r="W9" s="4" t="n">
-        <v>5</v>
+        <v>121</v>
       </c>
       <c r="X9" s="4" t="inlineStr">
         <is>
-          <t>锁定落点；半径1.5m；每技能冷却2s</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>移动散射(3发)</t>
+        </is>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA9" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" s="3">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>M_FOX_Dash</t>
@@ -2314,11 +2381,20 @@
           <t>预警0.8s；长4.5m宽1.4m；冷却4s</t>
         </is>
       </c>
-    </row>
-    <row r="11">
+      <c r="Y10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" s="3">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>M_RABBIT_MovingVolley</t>
+          <t>M_RABBIT_RangedBurst</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -2334,8 +2410,10 @@
       <c r="D11" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="4" t="b">
-        <v>1</v>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
       <c r="F11" s="4" t="n">
         <v>1</v>
@@ -2350,13 +2428,13 @@
         <v>0</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>1080</v>
+        <v>1000</v>
       </c>
       <c r="M11" s="4" t="n">
         <v>150</v>
@@ -2375,7 +2453,7 @@
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>LockedDirection</t>
+          <t>LockedLocation</t>
         </is>
       </c>
       <c r="S11" s="4" t="inlineStr">
@@ -2391,16 +2469,25 @@
       </c>
       <c r="V11" s="4" t="inlineStr">
         <is>
-          <t>全怪物技能表</t>
+          <t>怪物配置表</t>
         </is>
       </c>
       <c r="W11" s="4" t="n">
-        <v>121</v>
+        <v>5</v>
       </c>
       <c r="X11" s="4" t="inlineStr">
         <is>
-          <t>移动散射(3发)</t>
-        </is>
+          <t>锁定落点；半径1.5m；每技能冷却2s</t>
+        </is>
+      </c>
+      <c r="Y11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="4" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[PROGRAMMER] Integrate enemy presentation and approved assets
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="EnemyCombatStats" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyCombatStats" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -521,6 +521,13 @@
     <col width="13" customWidth="1" style="3" min="22" max="22"/>
     <col width="12" customWidth="1" style="3" min="23" max="23"/>
     <col width="12" customWidth="1" style="3" min="24" max="24"/>
+    <col width="13" customWidth="1" style="3" min="25" max="25"/>
+    <col width="13" customWidth="1" style="3" min="26" max="26"/>
+    <col width="13" customWidth="1" style="3" min="27" max="27"/>
+    <col width="13" customWidth="1" style="3" min="28" max="28"/>
+    <col width="13" customWidth="1" style="3" min="29" max="29"/>
+    <col width="13" customWidth="1" style="3" min="30" max="30"/>
+    <col width="13" customWidth="1" style="3" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -687,7 +694,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" s="3">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>M_Grunt</t>
@@ -798,7 +805,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" s="3">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>M_Shield</t>
@@ -909,7 +916,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" s="3">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>M_Bomber</t>
@@ -1020,7 +1027,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" s="3">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>M_SHEEP</t>
@@ -1135,7 +1142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" s="3">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>M_SLIME</t>
@@ -1225,7 +1232,7 @@
         </is>
       </c>
       <c r="Y8" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z8" s="4" t="n">
         <v>2000</v>
@@ -1244,7 +1251,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" s="3">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>M_RABBIT</t>
@@ -1334,7 +1341,7 @@
         </is>
       </c>
       <c r="Y9" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z9" s="4" t="n">
         <v>1500</v>
@@ -1353,7 +1360,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" s="3">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>M_FOX</t>
@@ -1443,7 +1450,7 @@
         </is>
       </c>
       <c r="Y10" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z10" s="4" t="n">
         <v>2000</v>

</xml_diff>

<commit_message>
[PROGRAMMER] Implement enemy time shard drops
Add the authoritative encounter reward table, death-time Run transaction, save migration, idempotence, tests, documentation, and refreshed Editor prebuilt bundle.
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyCombatStats" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="EnemyCombatStats" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:AE10" headerRowCount="1" totalsRowCount="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblEnemies" displayName="tblEnemies" ref="A3:AD10" headerRowCount="1" totalsRowCount="0">
   <autoFilter ref="A3:X10"/>
   <tableColumns count="30">
     <tableColumn id="1" name="Id"/>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AD10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -537,6 +537,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -635,60 +636,55 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>Reward</t>
+          <t>Boss</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>Boss</t>
+          <t>SourceSheet</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>SourceSheet</t>
+          <t>SourceRow</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>SourceRow</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
           <t>Notes</t>
         </is>
       </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>Phase2Enabled</t>
+        </is>
+      </c>
       <c r="Y3" s="5" t="inlineStr">
         <is>
-          <t>Phase2Enabled</t>
+          <t>Phase2TriggerRangeCm</t>
         </is>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>Phase2TriggerRangeCm</t>
+          <t>Phase2RequiredAttackCount</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>Phase2RequiredAttackCount</t>
-        </is>
-      </c>
-      <c r="AB3" s="5" t="inlineStr">
-        <is>
           <t>Phase2TransformSeconds</t>
         </is>
       </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Phase2TriggerMode</t>
+        </is>
+      </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>Phase2TriggerMode</t>
+          <t>Phase2HealthThresholdRatio</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
-        <is>
-          <t>Phase2HealthThresholdRatio</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
         <is>
           <t>HateRangeCm</t>
         </is>
@@ -762,31 +758,31 @@
       <c r="S4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>1</v>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
+          <t>怪物体系M</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>基础近战怪</t>
+        </is>
+      </c>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>怪物体系M</t>
-        </is>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="X4" s="4" t="inlineStr">
-        <is>
-          <t>基础近战怪</t>
-        </is>
-      </c>
-      <c r="Y4" s="4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="Y4" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Z4" s="4" t="n">
         <v>0</v>
@@ -794,14 +790,11 @@
       <c r="AA4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AB4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="4" t="n"/>
+      <c r="AB4" s="4" t="n"/>
+      <c r="AC4" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -873,31 +866,31 @@
       <c r="S5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T5" s="4" t="n">
-        <v>2</v>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
+          <t>怪物体系M</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="W5" s="4" t="inlineStr">
+        <is>
+          <t>正面减伤盾怪</t>
+        </is>
+      </c>
+      <c r="X5" s="4" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>怪物体系M</t>
-        </is>
-      </c>
-      <c r="W5" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="X5" s="4" t="inlineStr">
-        <is>
-          <t>正面减伤盾怪</t>
-        </is>
-      </c>
-      <c r="Y5" s="4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="Y5" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Z5" s="4" t="n">
         <v>0</v>
@@ -905,14 +898,11 @@
       <c r="AA5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AB5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="4" t="n"/>
+      <c r="AB5" s="4" t="n"/>
+      <c r="AC5" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -984,31 +974,31 @@
       <c r="S6" s="4" t="n">
         <v>1.2</v>
       </c>
-      <c r="T6" s="4" t="n">
-        <v>2</v>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
+          <t>怪物体系M</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="W6" s="4" t="inlineStr">
+        <is>
+          <t>接近后引爆</t>
+        </is>
+      </c>
+      <c r="X6" s="4" t="inlineStr">
+        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>怪物体系M</t>
-        </is>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="X6" s="4" t="inlineStr">
-        <is>
-          <t>接近后引爆</t>
-        </is>
-      </c>
-      <c r="Y6" s="4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="Y6" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Z6" s="4" t="n">
         <v>0</v>
@@ -1016,14 +1006,11 @@
       <c r="AA6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AB6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="4" t="n"/>
+      <c r="AB6" s="4" t="n"/>
+      <c r="AC6" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" s="4" t="n">
         <v>520</v>
       </c>
     </row>
@@ -1095,50 +1082,47 @@
       <c r="S7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T7" s="4" t="n">
-        <v>30</v>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="W7" s="4" t="inlineStr">
+        <is>
+          <t>第八场羊Boss；平A+3技能，血条清空变身为黑色二阶段(650满血再战)，变身范围40m</t>
+        </is>
+      </c>
+      <c r="X7" s="4" t="inlineStr">
+        <is>
           <t>true</t>
         </is>
       </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>怪物配置表</t>
-        </is>
-      </c>
-      <c r="W7" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="X7" s="4" t="inlineStr">
-        <is>
-          <t>第八场羊Boss；平A+3技能，血条清空变身为黑色二阶段(650满血再战)，变身范围40m</t>
-        </is>
-      </c>
-      <c r="Y7" s="4" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="Y7" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Z7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC7" s="4" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="4" t="inlineStr">
         <is>
           <t>HealthThreshold</t>
         </is>
       </c>
+      <c r="AC7" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1210,44 +1194,41 @@
       <c r="S8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T8" s="4" t="n">
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="W8" s="4" t="inlineStr">
+        <is>
+          <t>开普勒近战史莱姆；接触攻击</t>
+        </is>
+      </c>
+      <c r="X8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Z8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>怪物配置表</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>开普勒近战史莱姆；接触攻击</t>
-        </is>
-      </c>
-      <c r="Y8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z8" s="4" t="n">
-        <v>2000</v>
-      </c>
       <c r="AA8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC8" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AB8" s="4" t="n"/>
+      <c r="AC8" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE8" s="4" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1319,44 +1300,41 @@
       <c r="S9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T9" s="4" t="n">
-        <v>3</v>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
           <t>怪物配置表</t>
         </is>
       </c>
-      <c r="W9" s="4" t="n">
+      <c r="V9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="X9" s="4" t="inlineStr">
+      <c r="W9" s="4" t="inlineStr">
         <is>
           <t>开普勒远程兔子；锁定位置范围攻击</t>
         </is>
       </c>
-      <c r="Y9" s="4" t="b">
-        <v>1</v>
+      <c r="X9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>1500</v>
       </c>
       <c r="Z9" s="4" t="n">
-        <v>1500</v>
+        <v>2</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC9" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AB9" s="4" t="n"/>
+      <c r="AC9" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE9" s="4" t="n">
         <v>1500</v>
       </c>
     </row>
@@ -1428,44 +1406,41 @@
       <c r="S10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T10" s="4" t="n">
-        <v>4</v>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
           <t>怪物配置表</t>
         </is>
       </c>
-      <c r="W10" s="4" t="n">
+      <c r="V10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="X10" s="4" t="inlineStr">
+      <c r="W10" s="4" t="inlineStr">
         <is>
           <t>开普勒精英狐狸；正面防御与直线突进</t>
         </is>
       </c>
-      <c r="Y10" s="4" t="b">
-        <v>1</v>
+      <c r="X10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>2000</v>
       </c>
       <c r="Z10" s="4" t="n">
-        <v>2000</v>
+        <v>2</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AB10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC10" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AB10" s="4" t="n"/>
+      <c r="AC10" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AD10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE10" s="4" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1487,7 +1462,7 @@
     <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="T4:T10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
@@ -1502,7 +1477,7 @@
     <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="T4:T10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
     <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
@@ -1517,7 +1492,7 @@
     <dataValidation sqref="E4:E10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="T4:T10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
[PROGRAMMER] Fix sheep boss skill timing and VFX anchors
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -2108,7 +2108,7 @@
         <v>2</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.15</v>
+        <v>3</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>1</v>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="X8" s="4" t="inlineStr">
         <is>
-          <t>祷告光束；16伤/次；二阶段24伤；蓄力2s；WindupStart锁定</t>
+          <t>祷告光束；16伤/次；二阶段24伤；蓄力2s；光束与伤害窗口3s；WindupStart锁定</t>
         </is>
       </c>
       <c r="Y8" s="4" t="n">

</xml_diff>

<commit_message>
[DESIGNER] v1.1 data updates
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyCombatStats" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Enemies" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="EnemyAbilities" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BossPhases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="_ExportMap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="EnemyCombatStats" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -692,754 +692,754 @@
     <row r="4" s="3">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_Grunt</t>
+          <t>M_Grunt</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grunt</t>
+          <t>Grunt</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Grunt</t>
+          <t>Enemy.Grunt</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Grunt</t>
+          <t>Enemy.Grunt</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F4" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="4" t="n">
         <v>0.452</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="4" t="n">
         <v>51.84</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="4" t="n">
         <v>183.6</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="4" t="n">
         <v>1.3</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="4" t="n">
         <v>360</v>
       </c>
-      <c r="P4" s="4">
+      <c r="P4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q4" s="4">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4">
+      <c r="Q4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t>false</t>
         </is>
       </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物体系M</t>
-        </is>
-      </c>
-      <c r="V4" s="4">
+          <t>怪物体系M</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>4</v>
       </c>
       <c r="W4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">基础近战怪</t>
+          <t>基础近战怪</t>
         </is>
       </c>
       <c r="X4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
-        </is>
-      </c>
-      <c r="Y4" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="4"/>
-      <c r="AC4" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="4">
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="4" t="n"/>
+      <c r="AC4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="4" t="n">
         <v>520</v>
       </c>
     </row>
     <row r="5" s="3">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_Shield</t>
+          <t>M_Shield</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shield</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Shield</t>
+          <t>Enemy.Shield</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Shield</t>
+          <t>Enemy.Shield</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F5" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="4" t="n">
         <v>0.238</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="4" t="n">
         <v>51.84</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="4" t="n">
         <v>183.6</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="N5" s="4">
+      <c r="N5" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="O5" s="4">
+      <c r="O5" s="4" t="n">
         <v>360</v>
       </c>
-      <c r="P5" s="4">
+      <c r="P5" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q5" s="4">
-        <v>0</v>
-      </c>
-      <c r="R5" s="4">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4">
+      <c r="Q5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t>false</t>
         </is>
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物体系M</t>
-        </is>
-      </c>
-      <c r="V5" s="4">
+          <t>怪物体系M</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="n">
         <v>5</v>
       </c>
       <c r="W5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">正面减伤盾怪</t>
+          <t>正面减伤盾怪</t>
         </is>
       </c>
       <c r="X5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
-        </is>
-      </c>
-      <c r="Y5" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="4"/>
-      <c r="AC5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="4">
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="4" t="n"/>
+      <c r="AC5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="4" t="n">
         <v>520</v>
       </c>
     </row>
     <row r="6" s="3">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_Bomber</t>
+          <t>M_Bomber</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bomber</t>
+          <t>Bomber</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Bomber</t>
+          <t>Enemy.Bomber</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Bomber</t>
+          <t>Enemy.Bomber</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F6" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
         <v>10.5</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="4" t="n">
         <v>0.833</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="4" t="n">
         <v>51.84</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="4" t="n">
         <v>183.6</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="K6" s="4">
-        <v>0</v>
-      </c>
-      <c r="L6" s="4">
-        <v>0</v>
-      </c>
-      <c r="M6" s="4">
-        <v>0</v>
-      </c>
-      <c r="N6" s="4">
+      <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="O6" s="4">
+      <c r="O6" s="4" t="n">
         <v>360</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q6" s="4">
+      <c r="Q6" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="R6" s="4">
+      <c r="R6" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="S6" s="4">
+      <c r="S6" s="4" t="n">
         <v>1.2</v>
       </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t>false</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物体系M</t>
-        </is>
-      </c>
-      <c r="V6" s="4">
+          <t>怪物体系M</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>6</v>
       </c>
       <c r="W6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">接近后引爆</t>
+          <t>接近后引爆</t>
         </is>
       </c>
       <c r="X6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
-        </is>
-      </c>
-      <c r="Y6" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="4"/>
-      <c r="AC6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="4">
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="4" t="n"/>
+      <c r="AC6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="4" t="n">
         <v>520</v>
       </c>
     </row>
     <row r="7" s="3">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP</t>
+          <t>M_SHEEP</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss</t>
+          <t>Boss</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss.TimeGuard</t>
+          <t>Boss.TimeGuard</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.TimeGuard</t>
+          <t>Enemy.TimeGuard</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F7" s="4">
-        <v>1000</v>
-      </c>
-      <c r="G7" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <v>1.2</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="4" t="n">
         <v>183.6</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="4">
-        <v>2</v>
-      </c>
-      <c r="L7" s="4">
+      <c r="K7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="N7" s="4">
+      <c r="N7" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="O7" s="4">
+      <c r="O7" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="P7" s="4">
+      <c r="P7" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q7" s="4">
-        <v>0</v>
-      </c>
-      <c r="R7" s="4">
-        <v>0</v>
-      </c>
-      <c r="S7" s="4">
+      <c r="Q7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
+          <t>true</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="V7" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="n">
         <v>8</v>
       </c>
       <c r="W7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">第八场羊Boss；平A+3技能，血条清空变身为黑色二阶段(500满血再战)，变身范围40m</t>
+          <t>第八场羊Boss；平A+3技能，血条清空变身为黑色二阶段(500满血再战)，变身范围40m</t>
         </is>
       </c>
       <c r="X7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="Y7" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="4" t="n">
         <v>1</v>
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">HealthThreshold</t>
-        </is>
-      </c>
-      <c r="AC7" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="4">
+          <t>HealthThreshold</t>
+        </is>
+      </c>
+      <c r="AC7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" s="3">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
+          <t>M_SLIME</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Slime</t>
+          <t>Slime</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Slime</t>
+          <t>Enemy.Slime</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Slime</t>
+          <t>Enemy.Slime</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F8" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="J8" s="4">
-        <v>2</v>
-      </c>
-      <c r="K8" s="4">
+      <c r="J8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>1.3</v>
       </c>
-      <c r="L8" s="4">
+      <c r="L8" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="N8" s="4">
+      <c r="N8" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="O8" s="4">
+      <c r="O8" s="4" t="n">
         <v>360</v>
       </c>
-      <c r="P8" s="4">
+      <c r="P8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q8" s="4">
-        <v>0</v>
-      </c>
-      <c r="R8" s="4">
-        <v>0</v>
-      </c>
-      <c r="S8" s="4">
+      <c r="Q8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t>false</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="V8" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="W8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">开普勒近战史莱姆；接触攻击</t>
+          <t>开普勒近战史莱姆；接触攻击</t>
         </is>
       </c>
       <c r="X8" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="Y8" s="4">
+      <c r="Y8" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="Z8" s="4">
-        <v>2</v>
-      </c>
-      <c r="AA8" s="4">
-        <v>1</v>
-      </c>
-      <c r="AB8" s="4"/>
-      <c r="AC8" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD8" s="4">
+      <c r="Z8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB8" s="4" t="n"/>
+      <c r="AC8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="4" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="9" s="3">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
+          <t>M_RABBIT</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ranged</t>
+          <t>Ranged</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Ranged</t>
+          <t>Enemy.Ranged</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Rabbit</t>
+          <t>Enemy.Rabbit</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F9" s="4">
-        <v>2</v>
-      </c>
-      <c r="G9" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="4" t="n">
         <v>85</v>
       </c>
-      <c r="J9" s="4">
-        <v>1</v>
-      </c>
-      <c r="K9" s="4">
-        <v>2</v>
-      </c>
-      <c r="L9" s="4">
-        <v>0</v>
-      </c>
-      <c r="M9" s="4">
+      <c r="J9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4" t="n">
         <v>650</v>
       </c>
-      <c r="N9" s="4">
+      <c r="N9" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="O9" s="4">
+      <c r="O9" s="4" t="n">
         <v>360</v>
       </c>
-      <c r="P9" s="4">
+      <c r="P9" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q9" s="4">
-        <v>0</v>
-      </c>
-      <c r="R9" s="4">
-        <v>0</v>
-      </c>
-      <c r="S9" s="4">
+      <c r="Q9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t>false</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="V9" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="V9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="W9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">开普勒远程兔子；锁定位置范围攻击</t>
+          <t>开普勒远程兔子；锁定位置范围攻击</t>
         </is>
       </c>
       <c r="X9" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="Y9" s="4">
+      <c r="Y9" s="4" t="n">
         <v>900</v>
       </c>
-      <c r="Z9" s="4">
-        <v>2</v>
-      </c>
-      <c r="AA9" s="4">
-        <v>1</v>
-      </c>
-      <c r="AB9" s="4"/>
-      <c r="AC9" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="4">
+      <c r="Z9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="4" t="n"/>
+      <c r="AC9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="4" t="n">
         <v>900</v>
       </c>
     </row>
     <row r="10" s="3">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
+          <t>M_FOX</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elite</t>
+          <t>Elite</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Elite</t>
+          <t>Enemy.Elite</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.Fox</t>
+          <t>Enemy.Fox</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F10" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="4" t="n">
         <v>1.2</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="4" t="n">
         <v>130</v>
       </c>
-      <c r="J10" s="4">
-        <v>2</v>
-      </c>
-      <c r="K10" s="4">
+      <c r="J10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="4" t="n">
         <v>450</v>
       </c>
-      <c r="M10" s="4">
+      <c r="M10" s="4" t="n">
         <v>400</v>
       </c>
-      <c r="N10" s="4">
+      <c r="N10" s="4" t="n">
         <v>0.22</v>
       </c>
-      <c r="O10" s="4">
+      <c r="O10" s="4" t="n">
         <v>360</v>
       </c>
-      <c r="P10" s="4">
+      <c r="P10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q10" s="4">
-        <v>0</v>
-      </c>
-      <c r="R10" s="4">
-        <v>0</v>
-      </c>
-      <c r="S10" s="4">
+      <c r="Q10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">false</t>
+          <t>false</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="V10" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="V10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="W10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">开普勒精英狐狸；正面防御与直线突进</t>
+          <t>开普勒精英狐狸；正面防御与直线突进</t>
         </is>
       </c>
       <c r="X10" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="Y10" s="4">
+      <c r="Y10" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="Z10" s="4">
-        <v>2</v>
-      </c>
-      <c r="AA10" s="4">
-        <v>1</v>
-      </c>
-      <c r="AB10" s="4"/>
-      <c r="AC10" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD10" s="4">
+      <c r="Z10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB10" s="4" t="n"/>
+      <c r="AC10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="4" t="n">
         <v>1200</v>
       </c>
     </row>
@@ -1684,96 +1684,96 @@
     <row r="4" s="3">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP_MeleeSweep</t>
+          <t>M_SHEEP_MeleeSweep</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP</t>
+          <t>M_SHEEP</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss.MeleeSweep</t>
-        </is>
-      </c>
-      <c r="D4" s="4">
+          <t>Boss.MeleeSweep</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F4" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="4" t="n">
         <v>0.12</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K4" s="4">
-        <v>0</v>
-      </c>
-      <c r="L4" s="4">
+      <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="M4" s="4">
-        <v>0</v>
-      </c>
-      <c r="N4" s="4">
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>220</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="P4" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="4">
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedDirection</t>
+          <t>LockedDirection</t>
         </is>
       </c>
       <c r="S4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupStart</t>
-        </is>
-      </c>
-      <c r="T4" s="4">
-        <v>0</v>
-      </c>
-      <c r="U4" s="4">
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="W4" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="n">
         <v>8</v>
       </c>
       <c r="X4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">平A近战挥击；8伤；二阶段12伤；预警0.8s/收招0.5s</t>
-        </is>
-      </c>
-      <c r="Y4" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z4" s="4">
+          <t>平A近战挥击；8伤；二阶段12伤；预警0.8s/收招0.5s</t>
+        </is>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AA4" s="4" t="b">
@@ -1783,96 +1783,96 @@
     <row r="5" s="3">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP_StationaryVolley</t>
+          <t>M_SHEEP_StationaryVolley</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP</t>
+          <t>M_SHEEP</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss.Projectile</t>
-        </is>
-      </c>
-      <c r="D5" s="4">
+          <t>Boss.Projectile</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F5" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="H5" s="4">
-        <v>0</v>
-      </c>
-      <c r="I5" s="4">
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N5" s="4">
-        <v>0</v>
-      </c>
-      <c r="O5" s="4">
-        <v>0</v>
-      </c>
-      <c r="P5" s="4">
+      <c r="N5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="4" t="n">
         <v>840</v>
       </c>
-      <c r="Q5" s="4">
+      <c r="Q5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedLocation</t>
+          <t>LockedLocation</t>
         </is>
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupEnd</t>
-        </is>
-      </c>
-      <c r="T5" s="4">
-        <v>0</v>
-      </c>
-      <c r="U5" s="4">
+          <t>WindupEnd</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="W5" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="n">
         <v>8</v>
       </c>
       <c r="X5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">站定连射4连法杖弹；单发4伤总计16；二阶段总伤24；预警0.8s/收招0.5s</t>
-        </is>
-      </c>
-      <c r="Y5" s="4">
+          <t>站定连射4连法杖弹；单发4伤总计16；二阶段总伤24；预警0.8s/收招0.5s</t>
+        </is>
+      </c>
+      <c r="Y5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="Z5" s="4">
+      <c r="Z5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AA5" s="4" t="b">
@@ -1882,96 +1882,96 @@
     <row r="6" s="3">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP_MovingSpread</t>
+          <t>M_SHEEP_MovingSpread</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP</t>
+          <t>M_SHEEP</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss.Projectile</t>
-        </is>
-      </c>
-      <c r="D6" s="4">
+          <t>Boss.Projectile</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F6" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="H6" s="4">
-        <v>0</v>
-      </c>
-      <c r="I6" s="4">
-        <v>0</v>
-      </c>
-      <c r="J6" s="4">
-        <v>2</v>
-      </c>
-      <c r="K6" s="4">
+      <c r="H6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N6" s="4">
-        <v>0</v>
-      </c>
-      <c r="O6" s="4">
-        <v>0</v>
-      </c>
-      <c r="P6" s="4">
+      <c r="N6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>840</v>
       </c>
-      <c r="Q6" s="4">
+      <c r="Q6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedLocation</t>
+          <t>LockedLocation</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupStart</t>
-        </is>
-      </c>
-      <c r="T6" s="4">
-        <v>0</v>
-      </c>
-      <c r="U6" s="4">
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="W6" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="X6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">移动散射3向法杖弹；单发4伤总计12；二阶段总伤18；预警0.8s/无收招</t>
-        </is>
-      </c>
-      <c r="Y6" s="4">
+          <t>移动散射3向法杖弹；单发4伤总计12；二阶段总伤18；预警0.8s/无收招</t>
+        </is>
+      </c>
+      <c r="Y6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="Z6" s="4">
+      <c r="Z6" s="4" t="n">
         <v>40</v>
       </c>
       <c r="AA6" s="4" t="b">
@@ -1981,96 +1981,96 @@
     <row r="7" s="3">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP_BlinkSlam</t>
+          <t>M_SHEEP_BlinkSlam</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP</t>
+          <t>M_SHEEP</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss.BlinkSlam</t>
-        </is>
-      </c>
-      <c r="D7" s="4">
+          <t>Boss.BlinkSlam</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F7" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="4" t="n">
         <v>0.35</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K7" s="4">
-        <v>0</v>
-      </c>
-      <c r="L7" s="4">
+      <c r="K7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="N7" s="4">
-        <v>0</v>
-      </c>
-      <c r="O7" s="4">
-        <v>0</v>
-      </c>
-      <c r="P7" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="4">
+      <c r="N7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="n">
         <v>180</v>
       </c>
       <c r="R7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedLocation</t>
+          <t>LockedLocation</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupStart</t>
-        </is>
-      </c>
-      <c r="T7" s="4">
-        <v>0</v>
-      </c>
-      <c r="U7" s="4">
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="W7" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="n">
         <v>8</v>
       </c>
       <c r="X7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">闪身打击；24伤；二阶段36伤；收招0.5s</t>
-        </is>
-      </c>
-      <c r="Y7" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z7" s="4">
+          <t>闪身打击；24伤；二阶段36伤；收招0.5s</t>
+        </is>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AA7" s="4" t="b">
@@ -2080,96 +2080,96 @@
     <row r="8" s="3">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP_PrayerBeam</t>
+          <t>M_SHEEP_PrayerBeam</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SHEEP</t>
+          <t>M_SHEEP</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Boss.PrayerBeam</t>
-        </is>
-      </c>
-      <c r="D8" s="4">
+          <t>Boss.PrayerBeam</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F8" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="G8" s="4">
-        <v>2</v>
-      </c>
-      <c r="H8" s="4">
+      <c r="G8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I8" s="4">
-        <v>1</v>
-      </c>
-      <c r="J8" s="4">
+      <c r="I8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="K8" s="4">
-        <v>0</v>
-      </c>
-      <c r="L8" s="4">
+      <c r="K8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>2000</v>
       </c>
-      <c r="M8" s="4">
-        <v>0</v>
-      </c>
-      <c r="N8" s="4">
+      <c r="M8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>160</v>
       </c>
-      <c r="O8" s="4">
+      <c r="O8" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="P8" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="4">
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedDirection</t>
+          <t>LockedDirection</t>
         </is>
       </c>
       <c r="S8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupStart</t>
-        </is>
-      </c>
-      <c r="T8" s="4">
-        <v>0</v>
-      </c>
-      <c r="U8" s="4">
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="W8" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="X8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">祷告光束；16伤/次；二阶段24伤；蓄力2s；光束与伤害窗口3s；WindupStart锁定</t>
-        </is>
-      </c>
-      <c r="Y8" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z8" s="4">
+          <t>祷告光束；16伤/次；二阶段24伤；蓄力2s；光束与伤害窗口3s；WindupStart锁定</t>
+        </is>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AA8" s="4" t="b">
@@ -2179,94 +2179,94 @@
     <row r="9" s="3">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_MovingVolley</t>
+          <t>M_RABBIT_MovingVolley</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
+          <t>M_RABBIT</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.RangedBurst</t>
-        </is>
-      </c>
-      <c r="D9" s="4">
+          <t>Enemy.RangedBurst</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="F9" s="4">
-        <v>1</v>
-      </c>
-      <c r="G9" s="4">
+      <c r="F9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>0.55</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="4" t="n">
         <v>0.1</v>
       </c>
-      <c r="I9" s="4">
-        <v>0</v>
-      </c>
-      <c r="J9" s="4">
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
         <v>1.6</v>
       </c>
-      <c r="K9" s="4">
-        <v>0</v>
-      </c>
-      <c r="L9" s="4">
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
         <v>1080</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N9" s="4">
-        <v>0</v>
-      </c>
-      <c r="O9" s="4">
-        <v>0</v>
-      </c>
-      <c r="P9" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="4">
+      <c r="N9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedDirection</t>
+          <t>LockedDirection</t>
         </is>
       </c>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupStart</t>
-        </is>
-      </c>
-      <c r="T9" s="4">
-        <v>0</v>
-      </c>
-      <c r="U9" s="4">
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">全怪物技能表</t>
-        </is>
-      </c>
-      <c r="W9" s="4">
+          <t>全怪物技能表</t>
+        </is>
+      </c>
+      <c r="W9" s="4" t="n">
         <v>121</v>
       </c>
       <c r="X9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">移动散射(3发)</t>
-        </is>
-      </c>
-      <c r="Y9" s="4">
+          <t>移动散射(3发)</t>
+        </is>
+      </c>
+      <c r="Y9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="Z9" s="4">
+      <c r="Z9" s="4" t="n">
         <v>40</v>
       </c>
       <c r="AA9" s="4" t="b">
@@ -2276,96 +2276,96 @@
     <row r="10" s="3">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_Dash</t>
+          <t>M_FOX_Dash</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
+          <t>M_FOX</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.EliteDash</t>
-        </is>
-      </c>
-      <c r="D10" s="4">
+          <t>Enemy.EliteDash</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F10" s="4">
-        <v>2</v>
-      </c>
-      <c r="G10" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>0.8</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="4" t="n">
         <v>0.15</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="4" t="n">
         <v>2.5</v>
       </c>
-      <c r="K10" s="4">
-        <v>0</v>
-      </c>
-      <c r="L10" s="4">
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>650</v>
       </c>
-      <c r="M10" s="4">
-        <v>0</v>
-      </c>
-      <c r="N10" s="4">
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="O10" s="4">
+      <c r="O10" s="4" t="n">
         <v>650</v>
       </c>
-      <c r="P10" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="4">
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedDirection</t>
+          <t>LockedDirection</t>
         </is>
       </c>
       <c r="S10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupStart</t>
-        </is>
-      </c>
-      <c r="T10" s="4">
-        <v>0</v>
-      </c>
-      <c r="U10" s="4">
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="W10" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="X10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">预警0.8s；长6.5m宽1.4m；2伤；冷却2.5s</t>
-        </is>
-      </c>
-      <c r="Y10" s="4">
-        <v>1</v>
-      </c>
-      <c r="Z10" s="4">
+          <t>预警0.8s；长6.5m宽1.4m；2伤；冷却2.5s</t>
+        </is>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AA10" s="4" t="b">
@@ -2375,96 +2375,96 @@
     <row r="11" s="3">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_RangedBurst</t>
+          <t>M_RABBIT_RangedBurst</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
+          <t>M_RABBIT</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enemy.RangedBurst</t>
-        </is>
-      </c>
-      <c r="D11" s="4">
+          <t>Enemy.RangedBurst</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">true</t>
-        </is>
-      </c>
-      <c r="F11" s="4">
-        <v>1</v>
-      </c>
-      <c r="G11" s="4">
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4" t="n">
         <v>0.55</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="4" t="n">
         <v>0.35</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="4" t="n">
         <v>1.4</v>
       </c>
-      <c r="K11" s="4">
-        <v>0</v>
-      </c>
-      <c r="L11" s="4">
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M11" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="N11" s="4">
-        <v>0</v>
-      </c>
-      <c r="O11" s="4">
-        <v>0</v>
-      </c>
-      <c r="P11" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="4">
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LockedLocation</t>
+          <t>LockedLocation</t>
         </is>
       </c>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WindupStart</t>
-        </is>
-      </c>
-      <c r="T11" s="4">
-        <v>0</v>
-      </c>
-      <c r="U11" s="4">
+          <t>WindupStart</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="V11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">怪物配置表</t>
-        </is>
-      </c>
-      <c r="W11" s="4">
+          <t>怪物配置表</t>
+        </is>
+      </c>
+      <c r="W11" s="4" t="n">
         <v>5</v>
       </c>
       <c r="X11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">锁定落点；半径1m；预警0.55s/收招0.35s；冷却1.4s</t>
-        </is>
-      </c>
-      <c r="Y11" s="4">
+          <t>锁定落点；半径1m；预警0.55s/收招0.35s；冷却1.4s</t>
+        </is>
+      </c>
+      <c r="Y11" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="Z11" s="4">
+      <c r="Z11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AA11" s="4" t="b">
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="K5" s="4" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
@@ -3007,576 +3007,576 @@
     <row r="4" s="3">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C1</t>
+          <t>M_SLIME_C1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C4" s="4">
-        <v>1</v>
-      </c>
-      <c r="D4" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="4">
-        <v>2</v>
-      </c>
-      <c r="F4" s="4">
+      <c r="E4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="5" s="3">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C2</t>
+          <t>M_SLIME_C2</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C5" s="4">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="4">
-        <v>2</v>
-      </c>
-      <c r="F5" s="4">
+      <c r="E5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="6" s="3">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C3</t>
+          <t>M_SLIME_C3</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C6" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="4">
-        <v>2</v>
-      </c>
-      <c r="F6" s="4">
+      <c r="E6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="7" s="3">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C4</t>
+          <t>M_SLIME_C4</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C7" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="8" s="3">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C5</t>
+          <t>M_SLIME_C5</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C8" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="9" s="3">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C6</t>
+          <t>M_SLIME_C6</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C9" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="10" s="3">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C7</t>
+          <t>M_SLIME_C7</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C10" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="11" s="3">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME_C8</t>
+          <t>M_SLIME_C8</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_SLIME</t>
-        </is>
-      </c>
-      <c r="C11" s="4">
+          <t>M_SLIME</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
     <row r="12" s="3">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C1</t>
+          <t>M_RABBIT_C1</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C12" s="4">
-        <v>1</v>
-      </c>
-      <c r="D12" s="4">
-        <v>2</v>
-      </c>
-      <c r="E12" s="4">
-        <v>1</v>
-      </c>
-      <c r="F12" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13" s="3">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C2</t>
+          <t>M_RABBIT_C2</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C13" s="4">
-        <v>2</v>
-      </c>
-      <c r="D13" s="4">
-        <v>2</v>
-      </c>
-      <c r="E13" s="4">
-        <v>1</v>
-      </c>
-      <c r="F13" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="14" s="3">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C3</t>
+          <t>M_RABBIT_C3</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C14" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="4">
-        <v>2</v>
-      </c>
-      <c r="E14" s="4">
-        <v>1</v>
-      </c>
-      <c r="F14" s="4">
+      <c r="D14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15" s="3">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C4</t>
+          <t>M_RABBIT_C4</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C15" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="4">
-        <v>2</v>
-      </c>
-      <c r="E15" s="4">
-        <v>1</v>
-      </c>
-      <c r="F15" s="4">
+      <c r="D15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="16" s="3">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C5</t>
+          <t>M_RABBIT_C5</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C16" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E16" s="4">
-        <v>2</v>
-      </c>
-      <c r="F16" s="4">
+      <c r="E16" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17" s="3">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C6</t>
+          <t>M_RABBIT_C6</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C17" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E17" s="4">
-        <v>2</v>
-      </c>
-      <c r="F17" s="4">
+      <c r="E17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="18" s="3">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C7</t>
+          <t>M_RABBIT_C7</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C18" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E18" s="4">
-        <v>2</v>
-      </c>
-      <c r="F18" s="4">
+      <c r="E18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="19" s="3">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT_C8</t>
+          <t>M_RABBIT_C8</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_RABBIT</t>
-        </is>
-      </c>
-      <c r="C19" s="4">
+          <t>M_RABBIT</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E19" s="4">
-        <v>2</v>
-      </c>
-      <c r="F19" s="4">
+      <c r="E19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="20" s="3">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C1</t>
+          <t>M_FOX_C1</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C20" s="4">
-        <v>1</v>
-      </c>
-      <c r="D20" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E20" s="4">
-        <v>2</v>
-      </c>
-      <c r="F20" s="4">
+      <c r="E20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="21" s="3">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C2</t>
+          <t>M_FOX_C2</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C21" s="4">
-        <v>2</v>
-      </c>
-      <c r="D21" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E21" s="4">
-        <v>2</v>
-      </c>
-      <c r="F21" s="4">
+      <c r="E21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="22" s="3">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C3</t>
+          <t>M_FOX_C3</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C22" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="23" s="3">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C4</t>
+          <t>M_FOX_C4</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C23" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="24" s="3">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C5</t>
+          <t>M_FOX_C5</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C24" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="25" s="3">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C6</t>
+          <t>M_FOX_C6</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C25" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="26" s="3">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C7</t>
+          <t>M_FOX_C7</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C26" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="27" s="3">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX_C8</t>
+          <t>M_FOX_C8</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">M_FOX</t>
-        </is>
-      </c>
-      <c r="C27" s="4">
+          <t>M_FOX</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="4" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[PROGRAMMER] fix easter echoes and enemy health
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEnemyData.xlsx
+++ b/Design/Data/ReEchoEnemyData.xlsx
@@ -489,12 +489,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF12"/>
+  <dimension ref="A1:AD10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -537,7 +537,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1688,17 +1687,11 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:X1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
   <dataValidations count="15">
     <dataValidation sqref="B4:B10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Grunt,Shield,Bomber,Boss"</formula1>
@@ -1746,16 +1739,20 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC13"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -1791,7 +1788,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2993,17 +2989,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:X1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
   <dataValidations count="15">
     <dataValidation sqref="C4:C11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Boss.MeleeSweep,Boss.Projectile,Boss.BlinkSlam,Boss.PrayerBeam,Boss.ElementCleanse"</formula1>
@@ -3051,16 +3041,20 @@
       <formula1>"WindupStart,WindupEnd,Interval"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="1"/>
@@ -3086,7 +3080,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -3290,10 +3283,8 @@
           <t>RefillToMaximum</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
+      <c r="K5" s="4" t="n">
+        <v>2000000</v>
       </c>
       <c r="L5" s="4" t="b">
         <v>1</v>
@@ -3314,17 +3305,11 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
   <dataValidations count="12">
     <dataValidation sqref="E4:E5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"DestroyEncounterEchoes"</formula1>
@@ -3363,6 +3348,10 @@
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3517,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3527,7 +3516,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -3704,10 +3692,8 @@
           <t>5</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="D8" s="4" t="n">
+        <v>20000</v>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
@@ -3736,10 +3722,8 @@
           <t>6</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="D9" s="4" t="n">
+        <v>50000</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
@@ -3768,10 +3752,8 @@
           <t>7</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="D10" s="4" t="n">
+        <v>200000</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
@@ -3800,10 +3782,8 @@
           <t>8</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="D11" s="4" t="n">
+        <v>500000</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
@@ -3960,10 +3940,8 @@
           <t>5</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="D16" s="4" t="n">
+        <v>20000</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
@@ -3992,10 +3970,8 @@
           <t>6</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="D17" s="4" t="n">
+        <v>50000</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
@@ -4024,10 +4000,8 @@
           <t>7</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="D18" s="4" t="n">
+        <v>200000</v>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
@@ -4056,10 +4030,8 @@
           <t>8</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="D19" s="4" t="n">
+        <v>500000</v>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
@@ -4216,10 +4188,8 @@
           <t>5</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="D24" s="4" t="n">
+        <v>20000</v>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
@@ -4248,10 +4218,8 @@
           <t>6</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
+      <c r="D25" s="4" t="n">
+        <v>50000</v>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
@@ -4280,10 +4248,8 @@
           <t>7</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>140</t>
-        </is>
+      <c r="D26" s="4" t="n">
+        <v>200000</v>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
@@ -4312,10 +4278,8 @@
           <t>8</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
+      <c r="D27" s="4" t="n">
+        <v>500000</v>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
@@ -4328,8 +4292,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>